<commit_message>
update growth rate assumption
</commit_message>
<xml_diff>
--- a/lumen-saas-model.xlsx
+++ b/lumen-saas-model.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="131">
   <si>
     <t xml:space="preserve">Lumen Analytics · SaaS Financial Model</t>
   </si>
@@ -44,7 +44,7 @@
     <t xml:space="preserve">acquisition, retention, ACV, opex ratios) translate into ARR, revenue,</t>
   </si>
   <si>
-    <t xml:space="preserve">and operating margin across Base / Bull / Bear scenarios.</t>
+    <t xml:space="preserve">and operating margin across Base / Upside / Downside scenarios.</t>
   </si>
   <si>
     <t xml:space="preserve">How to use:</t>
@@ -53,7 +53,7 @@
     <t xml:space="preserve">  1. Open the Assumptions tab.</t>
   </si>
   <si>
-    <t xml:space="preserve">  2. Change the scenario toggle (cell C3) to 1 (Base), 2 (Bull), or 3 (Bear).</t>
+    <t xml:space="preserve">  2. Change the scenario toggle (cell C3) — pick Base, Upside, or Downside from the dropdown.</t>
   </si>
   <si>
     <t xml:space="preserve">  3. All downstream metrics on Revenue, P&amp;L, and Summary recalculate.</t>
@@ -188,31 +188,34 @@
     <t xml:space="preserve">Illustrative model. Synthetic data for portfolio demonstration.</t>
   </si>
   <si>
-    <t xml:space="preserve">Toggle scenario on Assumptions!C3 (1=Base, 2=Bull, 3=Bear) — all downstream metrics update.</t>
+    <t xml:space="preserve">Toggle scenario via the Base / Upside / Downside dropdown on Assumptions!C3 — all downstream metrics update.</t>
   </si>
   <si>
     <t xml:space="preserve">Lumen Analytics · Driver Assumptions</t>
   </si>
   <si>
-    <t xml:space="preserve">Scenario (1=Base, 2=Bull, 3=Bear)</t>
+    <t xml:space="preserve">Base</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario table</t>
   </si>
   <si>
-    <t xml:space="preserve">Base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bull</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bear</t>
+    <t xml:space="preserve">Upside</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Downside</t>
   </si>
   <si>
     <t xml:space="preserve">Starting customers</t>
   </si>
   <si>
     <t xml:space="preserve">New customers · Y1 quarterly growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New customers · Y2 quarterly growth</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New customers · Y3 quarterly growth</t>
   </si>
   <si>
     <t xml:space="preserve">Starting new customers / qtr</t>
@@ -1319,7 +1322,7 @@
         <v>21</v>
       </c>
       <c r="C3" s="5" t="str">
-        <f aca="false">CHOOSE(Scenario,"Base case","Bull case","Bear case")</f>
+        <f aca="false">Scenario&amp;" case"</f>
         <v>Base case</v>
       </c>
       <c r="D3" s="6" t="s">
@@ -1529,7 +1532,7 @@
         <v>38</v>
       </c>
       <c r="C16" s="19" t="n">
-        <f aca="false">Assumptions!$C$28</f>
+        <f aca="false">Assumptions!$C$32</f>
         <v>1.15</v>
       </c>
       <c r="D16" s="6" t="s">
@@ -1541,7 +1544,7 @@
         <v>40</v>
       </c>
       <c r="C17" s="19" t="n">
-        <f aca="false">Assumptions!$C$27</f>
+        <f aca="false">Assumptions!$C$31</f>
         <v>0.92</v>
       </c>
       <c r="D17" s="6" t="s">
@@ -1553,7 +1556,7 @@
         <v>42</v>
       </c>
       <c r="C18" s="20" t="n">
-        <f aca="false">Assumptions!$C$38</f>
+        <f aca="false">Assumptions!$C$42</f>
         <v>11500</v>
       </c>
       <c r="D18" s="6" t="s">
@@ -1565,7 +1568,7 @@
         <v>44</v>
       </c>
       <c r="C19" s="21" t="n">
-        <f aca="false">IFERROR(Assumptions!$C$38/(Assumptions!C43*Assumptions!$C$29/12),0)</f>
+        <f aca="false">IFERROR(Assumptions!$C$42/(Assumptions!C47*Assumptions!$C$33/12),0)</f>
         <v>12.6373626373626</v>
       </c>
       <c r="D19" s="6" t="s">
@@ -1577,7 +1580,7 @@
         <v>46</v>
       </c>
       <c r="C20" s="20" t="n">
-        <f aca="false">IFERROR(Assumptions!C43*Assumptions!$C$29/(1-Assumptions!$C$27),0)</f>
+        <f aca="false">IFERROR(Assumptions!C47*Assumptions!$C$33/(1-Assumptions!$C$31),0)</f>
         <v>136500</v>
       </c>
       <c r="D20" s="6" t="s">
@@ -1589,7 +1592,7 @@
         <v>48</v>
       </c>
       <c r="C21" s="22" t="n">
-        <f aca="false">IFERROR((Assumptions!C43*Assumptions!$C$29/(1-Assumptions!$C$27))/Assumptions!$C$38,0)</f>
+        <f aca="false">IFERROR((Assumptions!C47*Assumptions!$C$33/(1-Assumptions!$C$31))/Assumptions!$C$42,0)</f>
         <v>11.8695652173913</v>
       </c>
       <c r="D21" s="6" t="s">
@@ -1637,7 +1640,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P50"/>
+  <dimension ref="A1:P54"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="38"/>
@@ -1666,10 +1669,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="23" t="s">
         <v>55</v>
-      </c>
-      <c r="C3" s="23" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1679,18 +1682,18 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C6" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="D6" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="24" t="s">
+      <c r="E6" s="24" t="s">
         <v>58</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C7" s="25" t="n">
         <v>150</v>
@@ -1704,7 +1707,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C8" s="26" t="n">
         <v>0.12</v>
@@ -1718,807 +1721,859 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="25" t="n">
-        <v>45</v>
-      </c>
-      <c r="D9" s="25" t="n">
-        <v>50</v>
-      </c>
-      <c r="E9" s="25" t="n">
-        <v>35</v>
+        <v>61</v>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E9" s="26" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="C10" s="26" t="n">
-        <v>0.92</v>
+        <v>0.07</v>
       </c>
       <c r="D10" s="26" t="n">
-        <v>0.94</v>
+        <v>0.09</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>0.88</v>
+        <v>0.03</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="C11" s="26" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="D11" s="26" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="E11" s="26" t="n">
-        <v>1.05</v>
+        <v>63</v>
+      </c>
+      <c r="C11" s="25" t="n">
+        <v>45</v>
+      </c>
+      <c r="D11" s="25" t="n">
+        <v>50</v>
+      </c>
+      <c r="E11" s="25" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="C12" s="26" t="n">
-        <v>0.78</v>
+        <v>0.92</v>
       </c>
       <c r="D12" s="26" t="n">
-        <v>0.8</v>
+        <v>0.94</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>0.75</v>
+        <v>0.88</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>63</v>
+        <v>38</v>
       </c>
       <c r="C13" s="26" t="n">
-        <v>0.48</v>
+        <v>1.15</v>
       </c>
       <c r="D13" s="26" t="n">
-        <v>0.42</v>
+        <v>1.25</v>
       </c>
       <c r="E13" s="26" t="n">
-        <v>0.55</v>
+        <v>1.05</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="C14" s="26" t="n">
-        <v>0.34</v>
+        <v>0.78</v>
       </c>
       <c r="D14" s="26" t="n">
-        <v>0.28</v>
+        <v>0.8</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>0.42</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C15" s="26" t="n">
-        <v>0.3</v>
+        <v>0.48</v>
       </c>
       <c r="D15" s="26" t="n">
-        <v>0.26</v>
+        <v>0.42</v>
       </c>
       <c r="E15" s="26" t="n">
-        <v>0.34</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>0.22</v>
+        <v>0.34</v>
       </c>
       <c r="D16" s="26" t="n">
-        <v>0.2</v>
+        <v>0.28</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>0.26</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C17" s="26" t="n">
-        <v>0.14</v>
+        <v>0.3</v>
       </c>
       <c r="D17" s="26" t="n">
-        <v>0.12</v>
+        <v>0.26</v>
       </c>
       <c r="E17" s="26" t="n">
-        <v>0.16</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C18" s="26" t="n">
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="D18" s="26" t="n">
-        <v>0.09</v>
+        <v>0.2</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>0.13</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C19" s="27" t="n">
-        <v>14000</v>
-      </c>
-      <c r="D19" s="27" t="n">
-        <v>15500</v>
-      </c>
-      <c r="E19" s="27" t="n">
-        <v>12500</v>
+        <v>68</v>
+      </c>
+      <c r="C19" s="26" t="n">
+        <v>0.14</v>
+      </c>
+      <c r="D19" s="26" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <v>0.16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C20" s="26" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="D20" s="26" t="n">
-        <v>0.07</v>
+        <v>0.09</v>
       </c>
       <c r="E20" s="26" t="n">
-        <v>0.03</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C21" s="27" t="n">
+        <v>14000</v>
+      </c>
+      <c r="D21" s="27" t="n">
+        <v>15500</v>
+      </c>
+      <c r="E21" s="27" t="n">
+        <v>12500</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C21" s="27" t="n">
+      <c r="C22" s="26" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D22" s="26" t="n">
+        <v>0.07</v>
+      </c>
+      <c r="E22" s="26" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C23" s="27" t="n">
         <v>11500</v>
       </c>
-      <c r="D21" s="27" t="n">
+      <c r="D23" s="27" t="n">
         <v>10500</v>
       </c>
-      <c r="E21" s="27" t="n">
+      <c r="E23" s="27" t="n">
         <v>13000</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="14" t="s">
-        <v>60</v>
-      </c>
-      <c r="C24" s="28" t="n">
-        <f aca="false">INDEX(C7:E7,Scenario)</f>
-        <v>150</v>
-      </c>
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="29" t="n">
-        <f aca="false">INDEX(C8:E8,Scenario)</f>
-        <v>0.12</v>
+      <c r="A25" s="2" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C26" s="28" t="n">
-        <f aca="false">INDEX(C9:E9,Scenario)</f>
-        <v>45</v>
+        <f aca="false">INDEX(C7:E7,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>150</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C27" s="29" t="n">
-        <f aca="false">INDEX(C10:E10,Scenario)</f>
-        <v>0.92</v>
+        <f aca="false">INDEX(C8:E8,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.12</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="C28" s="29" t="n">
-        <f aca="false">INDEX(C11:E11,Scenario)</f>
-        <v>1.15</v>
+        <f aca="false">INDEX(C9:E9,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.09</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="C29" s="29" t="n">
-        <f aca="false">INDEX(C12:E12,Scenario)</f>
-        <v>0.78</v>
+        <f aca="false">INDEX(C10:E10,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.07</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="29" t="n">
-        <f aca="false">INDEX(C13:E13,Scenario)</f>
-        <v>0.48</v>
+      <c r="C30" s="28" t="n">
+        <f aca="false">INDEX(C11:E11,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>45</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>64</v>
+        <v>40</v>
       </c>
       <c r="C31" s="29" t="n">
-        <f aca="false">INDEX(C14:E14,Scenario)</f>
-        <v>0.34</v>
+        <f aca="false">INDEX(C12:E12,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.92</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="14" t="s">
-        <v>65</v>
+        <v>38</v>
       </c>
       <c r="C32" s="29" t="n">
-        <f aca="false">INDEX(C15:E15,Scenario)</f>
-        <v>0.3</v>
+        <f aca="false">INDEX(C13:E13,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>1.15</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="14" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="C33" s="29" t="n">
-        <f aca="false">INDEX(C16:E16,Scenario)</f>
-        <v>0.22</v>
+        <f aca="false">INDEX(C14:E14,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.78</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C34" s="29" t="n">
-        <f aca="false">INDEX(C17:E17,Scenario)</f>
-        <v>0.14</v>
+        <f aca="false">INDEX(C15:E15,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.48</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C35" s="29" t="n">
-        <f aca="false">INDEX(C18:E18,Scenario)</f>
-        <v>0.1</v>
+        <f aca="false">INDEX(C16:E16,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.34</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C36" s="30" t="n">
-        <f aca="false">INDEX(C19:E19,Scenario)</f>
-        <v>14000</v>
+        <v>66</v>
+      </c>
+      <c r="C36" s="29" t="n">
+        <f aca="false">INDEX(C17:E17,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.3</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C37" s="29" t="n">
-        <f aca="false">INDEX(C20:E20,Scenario)</f>
-        <v>0.05</v>
+        <f aca="false">INDEX(C18:E18,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.22</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="C38" s="29" t="n">
+        <f aca="false">INDEX(C19:E19,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.14</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39" s="29" t="n">
+        <f aca="false">INDEX(C20:E20,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C40" s="30" t="n">
+        <f aca="false">INDEX(C21:E21,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="C38" s="30" t="n">
-        <f aca="false">INDEX(C21:E21,Scenario)</f>
-        <v>11500</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="2" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="11"/>
-      <c r="B41" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="C41" s="31" t="s">
-        <v>75</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="E41" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="F41" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="G41" s="31" t="s">
-        <v>79</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="I41" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="J41" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="K41" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="L41" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="M41" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="N41" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="O41" s="10" t="s">
-        <v>87</v>
+      <c r="C41" s="29" t="n">
+        <f aca="false">INDEX(C22:E22,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>0.05</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C42" s="30" t="n">
+        <f aca="false">INDEX(C23:E23,MATCH(Scenario,$C$6:$E$6,0))</f>
+        <v>11500</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="11"/>
+      <c r="B45" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C45" s="31" t="s">
+        <v>76</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E45" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F45" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="G45" s="31" t="s">
+        <v>80</v>
+      </c>
+      <c r="H45" s="10" t="s">
+        <v>81</v>
+      </c>
+      <c r="I45" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="J45" s="10" t="s">
+        <v>83</v>
+      </c>
+      <c r="K45" s="31" t="s">
+        <v>84</v>
+      </c>
+      <c r="L45" s="10" t="s">
+        <v>85</v>
+      </c>
+      <c r="M45" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="N45" s="10" t="s">
+        <v>87</v>
+      </c>
+      <c r="O45" s="10" t="s">
         <v>88</v>
-      </c>
-      <c r="B42" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="C42" s="32" t="n">
-        <f aca="false">Assumptions!$C$26</f>
-        <v>45</v>
-      </c>
-      <c r="D42" s="32" t="n">
-        <f aca="false">C42*(1+Assumptions!$C$25)</f>
-        <v>50.4</v>
-      </c>
-      <c r="E42" s="32" t="n">
-        <f aca="false">D42*(1+Assumptions!$C$25)</f>
-        <v>56.448</v>
-      </c>
-      <c r="F42" s="32" t="n">
-        <f aca="false">E42*(1+Assumptions!$C$25)</f>
-        <v>63.22176</v>
-      </c>
-      <c r="G42" s="32" t="n">
-        <f aca="false">F42*1.09</f>
-        <v>68.9117184</v>
-      </c>
-      <c r="H42" s="32" t="n">
-        <f aca="false">G42*1.09</f>
-        <v>75.113773056</v>
-      </c>
-      <c r="I42" s="32" t="n">
-        <f aca="false">H42*1.09</f>
-        <v>81.87401263104</v>
-      </c>
-      <c r="J42" s="32" t="n">
-        <f aca="false">I42*1.09</f>
-        <v>89.2426737678336</v>
-      </c>
-      <c r="K42" s="32" t="n">
-        <f aca="false">J42*1.07</f>
-        <v>95.489660931582</v>
-      </c>
-      <c r="L42" s="32" t="n">
-        <f aca="false">K42*1.07</f>
-        <v>102.173937196793</v>
-      </c>
-      <c r="M42" s="32" t="n">
-        <f aca="false">L42*1.07</f>
-        <v>109.326112800568</v>
-      </c>
-      <c r="N42" s="32" t="n">
-        <f aca="false">M42*1.07</f>
-        <v>116.978940696608</v>
-      </c>
-      <c r="O42" s="33" t="n">
-        <f aca="false">SUM(C42:N42)</f>
-        <v>954.180589480425</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="B43" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="C43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^0</f>
-        <v>14000</v>
-      </c>
-      <c r="D43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^0</f>
-        <v>14000</v>
-      </c>
-      <c r="E43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^0</f>
-        <v>14000</v>
-      </c>
-      <c r="F43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^0</f>
-        <v>14000</v>
-      </c>
-      <c r="G43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^1</f>
-        <v>14700</v>
-      </c>
-      <c r="H43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^1</f>
-        <v>14700</v>
-      </c>
-      <c r="I43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^1</f>
-        <v>14700</v>
-      </c>
-      <c r="J43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^1</f>
-        <v>14700</v>
-      </c>
-      <c r="K43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^2</f>
-        <v>15435</v>
-      </c>
-      <c r="L43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^2</f>
-        <v>15435</v>
-      </c>
-      <c r="M43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^2</f>
-        <v>15435</v>
-      </c>
-      <c r="N43" s="34" t="n">
-        <f aca="false">Assumptions!$C$36*(1+Assumptions!$C$37)^2</f>
-        <v>15435</v>
-      </c>
-      <c r="O43" s="35" t="n">
-        <f aca="false">AVERAGE(C43:N43)</f>
-        <v>14711.6666666667</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="14" t="s">
-        <v>92</v>
-      </c>
-      <c r="B44" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="D44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="E44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="F44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="G44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="H44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="I44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="J44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="K44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="L44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="M44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-      <c r="N44" s="36" t="n">
-        <f aca="false">1-Assumptions!$C$27^(1/4)</f>
-        <v>0.0206296386644407</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="14" t="s">
-        <v>94</v>
-      </c>
-      <c r="B45" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="D45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="E45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="F45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="G45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="H45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="I45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="J45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="K45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="L45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="M45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
-      </c>
-      <c r="N45" s="36" t="n">
-        <f aca="false">Assumptions!$C$28^(1/4)-Assumptions!$C$27^(1/4)</f>
-        <v>0.0561877150060628</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="14" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*0/11</f>
-        <v>0.48</v>
-      </c>
-      <c r="D46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*1/11</f>
-        <v>0.467272727272727</v>
-      </c>
-      <c r="E46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*2/11</f>
-        <v>0.454545454545455</v>
-      </c>
-      <c r="F46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*3/11</f>
-        <v>0.441818181818182</v>
-      </c>
-      <c r="G46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*4/11</f>
-        <v>0.429090909090909</v>
-      </c>
-      <c r="H46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*5/11</f>
-        <v>0.416363636363636</v>
-      </c>
-      <c r="I46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*6/11</f>
-        <v>0.403636363636364</v>
-      </c>
-      <c r="J46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*7/11</f>
-        <v>0.390909090909091</v>
-      </c>
-      <c r="K46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*8/11</f>
-        <v>0.378181818181818</v>
-      </c>
-      <c r="L46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*9/11</f>
-        <v>0.365454545454546</v>
-      </c>
-      <c r="M46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*10/11</f>
-        <v>0.352727272727273</v>
-      </c>
-      <c r="N46" s="36" t="n">
-        <f aca="false">Assumptions!$C$30+(Assumptions!$C$31-Assumptions!$C$30)*11/11</f>
-        <v>0.34</v>
+        <v>90</v>
+      </c>
+      <c r="C46" s="32" t="n">
+        <f aca="false">Assumptions!$C$30</f>
+        <v>45</v>
+      </c>
+      <c r="D46" s="32" t="n">
+        <f aca="false">C46*(1+Assumptions!$C$27)</f>
+        <v>50.4</v>
+      </c>
+      <c r="E46" s="32" t="n">
+        <f aca="false">D46*(1+Assumptions!$C$27)</f>
+        <v>56.448</v>
+      </c>
+      <c r="F46" s="32" t="n">
+        <f aca="false">E46*(1+Assumptions!$C$27)</f>
+        <v>63.22176</v>
+      </c>
+      <c r="G46" s="32" t="n">
+        <f aca="false">F46*(1+Assumptions!$C$28)</f>
+        <v>68.9117184</v>
+      </c>
+      <c r="H46" s="32" t="n">
+        <f aca="false">G46*(1+Assumptions!$C$28)</f>
+        <v>75.113773056</v>
+      </c>
+      <c r="I46" s="32" t="n">
+        <f aca="false">H46*(1+Assumptions!$C$28)</f>
+        <v>81.87401263104</v>
+      </c>
+      <c r="J46" s="32" t="n">
+        <f aca="false">I46*(1+Assumptions!$C$28)</f>
+        <v>89.2426737678336</v>
+      </c>
+      <c r="K46" s="32" t="n">
+        <f aca="false">J46*(1+Assumptions!$C$29)</f>
+        <v>95.489660931582</v>
+      </c>
+      <c r="L46" s="32" t="n">
+        <f aca="false">K46*(1+Assumptions!$C$29)</f>
+        <v>102.173937196793</v>
+      </c>
+      <c r="M46" s="32" t="n">
+        <f aca="false">L46*(1+Assumptions!$C$29)</f>
+        <v>109.326112800568</v>
+      </c>
+      <c r="N46" s="32" t="n">
+        <f aca="false">M46*(1+Assumptions!$C$29)</f>
+        <v>116.978940696608</v>
+      </c>
+      <c r="O46" s="33" t="n">
+        <f aca="false">SUM(C46:N46)</f>
+        <v>954.180589480425</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="14" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*0/11</f>
-        <v>0.3</v>
-      </c>
-      <c r="D47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*1/11</f>
-        <v>0.292727272727273</v>
-      </c>
-      <c r="E47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*2/11</f>
-        <v>0.285454545454545</v>
-      </c>
-      <c r="F47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*3/11</f>
-        <v>0.278181818181818</v>
-      </c>
-      <c r="G47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*4/11</f>
-        <v>0.270909090909091</v>
-      </c>
-      <c r="H47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*5/11</f>
-        <v>0.263636363636364</v>
-      </c>
-      <c r="I47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*6/11</f>
-        <v>0.256363636363636</v>
-      </c>
-      <c r="J47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*7/11</f>
-        <v>0.249090909090909</v>
-      </c>
-      <c r="K47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*8/11</f>
-        <v>0.241818181818182</v>
-      </c>
-      <c r="L47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*9/11</f>
-        <v>0.234545454545455</v>
-      </c>
-      <c r="M47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*10/11</f>
-        <v>0.227272727272727</v>
-      </c>
-      <c r="N47" s="36" t="n">
-        <f aca="false">Assumptions!$C$32+(Assumptions!$C$33-Assumptions!$C$32)*11/11</f>
-        <v>0.22</v>
+        <v>92</v>
+      </c>
+      <c r="C47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^0</f>
+        <v>14000</v>
+      </c>
+      <c r="D47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^0</f>
+        <v>14000</v>
+      </c>
+      <c r="E47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^0</f>
+        <v>14000</v>
+      </c>
+      <c r="F47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^0</f>
+        <v>14000</v>
+      </c>
+      <c r="G47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^1</f>
+        <v>14700</v>
+      </c>
+      <c r="H47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^1</f>
+        <v>14700</v>
+      </c>
+      <c r="I47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^1</f>
+        <v>14700</v>
+      </c>
+      <c r="J47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^1</f>
+        <v>14700</v>
+      </c>
+      <c r="K47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^2</f>
+        <v>15435</v>
+      </c>
+      <c r="L47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^2</f>
+        <v>15435</v>
+      </c>
+      <c r="M47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^2</f>
+        <v>15435</v>
+      </c>
+      <c r="N47" s="34" t="n">
+        <f aca="false">Assumptions!$C$40*(1+Assumptions!$C$41)^2</f>
+        <v>15435</v>
+      </c>
+      <c r="O47" s="35" t="n">
+        <f aca="false">AVERAGE(C47:N47)</f>
+        <v>14711.6666666667</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="B48" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="D48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="E48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="F48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="G48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="H48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="I48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="J48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="K48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="L48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="M48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+      <c r="N48" s="36" t="n">
+        <f aca="false">1-Assumptions!$C$31^(1/4)</f>
+        <v>0.0206296386644407</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="B49" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="D49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="E49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="F49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="G49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="H49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="I49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="J49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="K49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="L49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="M49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+      <c r="N49" s="36" t="n">
+        <f aca="false">Assumptions!$C$32^(1/4)-Assumptions!$C$31^(1/4)</f>
+        <v>0.0561877150060628</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="B50" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*0/11</f>
+        <v>0.48</v>
+      </c>
+      <c r="D50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*1/11</f>
+        <v>0.467272727272727</v>
+      </c>
+      <c r="E50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*2/11</f>
+        <v>0.454545454545455</v>
+      </c>
+      <c r="F50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*3/11</f>
+        <v>0.441818181818182</v>
+      </c>
+      <c r="G50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*4/11</f>
+        <v>0.429090909090909</v>
+      </c>
+      <c r="H50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*5/11</f>
+        <v>0.416363636363636</v>
+      </c>
+      <c r="I50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*6/11</f>
+        <v>0.403636363636364</v>
+      </c>
+      <c r="J50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*7/11</f>
+        <v>0.390909090909091</v>
+      </c>
+      <c r="K50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*8/11</f>
+        <v>0.378181818181818</v>
+      </c>
+      <c r="L50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*9/11</f>
+        <v>0.365454545454546</v>
+      </c>
+      <c r="M50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*10/11</f>
+        <v>0.352727272727273</v>
+      </c>
+      <c r="N50" s="36" t="n">
+        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*11/11</f>
+        <v>0.34</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="14" t="s">
         <v>97</v>
       </c>
-      <c r="B48" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="C48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*0/11</f>
+      <c r="B51" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*0/11</f>
+        <v>0.3</v>
+      </c>
+      <c r="D51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*1/11</f>
+        <v>0.292727272727273</v>
+      </c>
+      <c r="E51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*2/11</f>
+        <v>0.285454545454545</v>
+      </c>
+      <c r="F51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*3/11</f>
+        <v>0.278181818181818</v>
+      </c>
+      <c r="G51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*4/11</f>
+        <v>0.270909090909091</v>
+      </c>
+      <c r="H51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*5/11</f>
+        <v>0.263636363636364</v>
+      </c>
+      <c r="I51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*6/11</f>
+        <v>0.256363636363636</v>
+      </c>
+      <c r="J51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*7/11</f>
+        <v>0.249090909090909</v>
+      </c>
+      <c r="K51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*8/11</f>
+        <v>0.241818181818182</v>
+      </c>
+      <c r="L51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*9/11</f>
+        <v>0.234545454545455</v>
+      </c>
+      <c r="M51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*10/11</f>
+        <v>0.227272727272727</v>
+      </c>
+      <c r="N51" s="36" t="n">
+        <f aca="false">Assumptions!$C$36+(Assumptions!$C$37-Assumptions!$C$36)*11/11</f>
+        <v>0.22</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="14" t="s">
+        <v>98</v>
+      </c>
+      <c r="B52" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*0/11</f>
         <v>0.14</v>
       </c>
-      <c r="D48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*1/11</f>
+      <c r="D52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*1/11</f>
         <v>0.136363636363636</v>
       </c>
-      <c r="E48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*2/11</f>
+      <c r="E52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*2/11</f>
         <v>0.132727272727273</v>
       </c>
-      <c r="F48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*3/11</f>
+      <c r="F52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*3/11</f>
         <v>0.129090909090909</v>
       </c>
-      <c r="G48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*4/11</f>
+      <c r="G52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*4/11</f>
         <v>0.125454545454545</v>
       </c>
-      <c r="H48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*5/11</f>
+      <c r="H52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*5/11</f>
         <v>0.121818181818182</v>
       </c>
-      <c r="I48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*6/11</f>
+      <c r="I52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*6/11</f>
         <v>0.118181818181818</v>
       </c>
-      <c r="J48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*7/11</f>
+      <c r="J52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*7/11</f>
         <v>0.114545454545455</v>
       </c>
-      <c r="K48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*8/11</f>
+      <c r="K52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*8/11</f>
         <v>0.110909090909091</v>
       </c>
-      <c r="L48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*9/11</f>
+      <c r="L52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*9/11</f>
         <v>0.107272727272727</v>
       </c>
-      <c r="M48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*10/11</f>
+      <c r="M52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*10/11</f>
         <v>0.103636363636364</v>
       </c>
-      <c r="N48" s="36" t="n">
-        <f aca="false">Assumptions!$C$34+(Assumptions!$C$35-Assumptions!$C$34)*11/11</f>
+      <c r="N52" s="36" t="n">
+        <f aca="false">Assumptions!$C$38+(Assumptions!$C$39-Assumptions!$C$38)*11/11</f>
         <v>0.1</v>
       </c>
     </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B50" s="4"/>
-      <c r="C50" s="4"/>
-      <c r="D50" s="4"/>
-      <c r="E50" s="4"/>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
-      <c r="H50" s="4"/>
-      <c r="I50" s="4"/>
-      <c r="J50" s="4"/>
-      <c r="K50" s="4"/>
-      <c r="L50" s="4"/>
-      <c r="M50" s="4"/>
-      <c r="N50" s="4"/>
-      <c r="O50" s="4"/>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B54" s="4"/>
+      <c r="C54" s="4"/>
+      <c r="D54" s="4"/>
+      <c r="E54" s="4"/>
+      <c r="F54" s="4"/>
+      <c r="G54" s="4"/>
+      <c r="H54" s="4"/>
+      <c r="I54" s="4"/>
+      <c r="J54" s="4"/>
+      <c r="K54" s="4"/>
+      <c r="L54" s="4"/>
+      <c r="M54" s="4"/>
+      <c r="N54" s="4"/>
+      <c r="O54" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:P1"/>
-    <mergeCell ref="A50:O50"/>
+    <mergeCell ref="A54:O54"/>
   </mergeCells>
+  <dataValidations count="1">
+    <dataValidation allowBlank="false" error="Pick Base, Upside, or Downside" errorStyle="stop" errorTitle="Invalid scenario" operator="between" prompt="Select a scenario from the dropdown" promptTitle="Scenario" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C3" type="list">
+      <formula1>"Base,Upside,Downside"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -2544,7 +2599,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2564,7 +2619,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B3" s="4"/>
       <c r="C3" s="4"/>
@@ -2583,7 +2638,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -2604,54 +2659,54 @@
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11"/>
       <c r="B6" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K6" s="31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L6" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N6" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O6" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C7" s="37" t="n">
-        <f aca="false">Assumptions!$C$24</f>
+        <f aca="false">Assumptions!$C$26</f>
         <v>150</v>
       </c>
       <c r="D7" s="32" t="n">
@@ -2701,54 +2756,54 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C8" s="37" t="n">
-        <f aca="false">Assumptions!C42</f>
+        <f aca="false">Assumptions!C46</f>
         <v>45</v>
       </c>
       <c r="D8" s="37" t="n">
-        <f aca="false">Assumptions!D42</f>
+        <f aca="false">Assumptions!D46</f>
         <v>50.4</v>
       </c>
       <c r="E8" s="37" t="n">
-        <f aca="false">Assumptions!E42</f>
+        <f aca="false">Assumptions!E46</f>
         <v>56.448</v>
       </c>
       <c r="F8" s="37" t="n">
-        <f aca="false">Assumptions!F42</f>
+        <f aca="false">Assumptions!F46</f>
         <v>63.22176</v>
       </c>
       <c r="G8" s="37" t="n">
-        <f aca="false">Assumptions!G42</f>
+        <f aca="false">Assumptions!G46</f>
         <v>68.9117184</v>
       </c>
       <c r="H8" s="37" t="n">
-        <f aca="false">Assumptions!H42</f>
+        <f aca="false">Assumptions!H46</f>
         <v>75.113773056</v>
       </c>
       <c r="I8" s="37" t="n">
-        <f aca="false">Assumptions!I42</f>
+        <f aca="false">Assumptions!I46</f>
         <v>81.87401263104</v>
       </c>
       <c r="J8" s="37" t="n">
-        <f aca="false">Assumptions!J42</f>
+        <f aca="false">Assumptions!J46</f>
         <v>89.2426737678336</v>
       </c>
       <c r="K8" s="37" t="n">
-        <f aca="false">Assumptions!K42</f>
+        <f aca="false">Assumptions!K46</f>
         <v>95.489660931582</v>
       </c>
       <c r="L8" s="37" t="n">
-        <f aca="false">Assumptions!L42</f>
+        <f aca="false">Assumptions!L46</f>
         <v>102.173937196793</v>
       </c>
       <c r="M8" s="37" t="n">
-        <f aca="false">Assumptions!M42</f>
+        <f aca="false">Assumptions!M46</f>
         <v>109.326112800568</v>
       </c>
       <c r="N8" s="37" t="n">
-        <f aca="false">Assumptions!N42</f>
+        <f aca="false">Assumptions!N46</f>
         <v>116.978940696608</v>
       </c>
       <c r="O8" s="33" t="n">
@@ -2758,54 +2813,54 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C9" s="32" t="n">
-        <f aca="false">-C7*Assumptions!C44</f>
+        <f aca="false">-C7*Assumptions!C48</f>
         <v>-3.0944457996661</v>
       </c>
       <c r="D9" s="32" t="n">
-        <f aca="false">-D7*Assumptions!D44</f>
+        <f aca="false">-D7*Assumptions!D48</f>
         <v>-3.95894224085212</v>
       </c>
       <c r="E9" s="32" t="n">
-        <f aca="false">-E7*Assumptions!E44</f>
+        <f aca="false">-E7*Assumptions!E48</f>
         <v>-4.91700448161776</v>
       </c>
       <c r="F9" s="32" t="n">
-        <f aca="false">-F7*Assumptions!F44</f>
+        <f aca="false">-F7*Assumptions!F48</f>
         <v>-5.9800702991809</v>
       </c>
       <c r="G9" s="32" t="n">
-        <f aca="false">-G7*Assumptions!G44</f>
+        <f aca="false">-G7*Assumptions!G48</f>
         <v>-7.16094567425084</v>
       </c>
       <c r="H9" s="32" t="n">
-        <f aca="false">-H7*Assumptions!H44</f>
+        <f aca="false">-H7*Assumptions!H48</f>
         <v>-8.43484180283304</v>
       </c>
       <c r="I9" s="32" t="n">
-        <f aca="false">-I7*Assumptions!I44</f>
+        <f aca="false">-I7*Assumptions!I48</f>
         <v>-9.81040406111695</v>
       </c>
       <c r="J9" s="32" t="n">
-        <f aca="false">-J7*Assumptions!J44</f>
+        <f aca="false">-J7*Assumptions!J48</f>
         <v>-11.2970502667702</v>
       </c>
       <c r="K9" s="32" t="n">
-        <f aca="false">-K7*Assumptions!K44</f>
+        <f aca="false">-K7*Assumptions!K48</f>
         <v>-12.9050403150716</v>
       </c>
       <c r="L9" s="32" t="n">
-        <f aca="false">-L7*Assumptions!L44</f>
+        <f aca="false">-L7*Assumptions!L48</f>
         <v>-14.6087311976302</v>
       </c>
       <c r="M9" s="32" t="n">
-        <f aca="false">-M7*Assumptions!M44</f>
+        <f aca="false">-M7*Assumptions!M48</f>
         <v>-16.4151697569702</v>
       </c>
       <c r="N9" s="32" t="n">
-        <f aca="false">-N7*Assumptions!N44</f>
+        <f aca="false">-N7*Assumptions!N48</f>
         <v>-18.3318889399321</v>
       </c>
       <c r="O9" s="33" t="n">
@@ -2872,7 +2927,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -2893,54 +2948,54 @@
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11"/>
       <c r="B14" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G14" s="31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K14" s="31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L14" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M14" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N14" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O14" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C15" s="39" t="n">
-        <f aca="false">Assumptions!$C$24*Assumptions!C43/1000</f>
+        <f aca="false">Assumptions!$C$26*Assumptions!C47/1000</f>
         <v>2100</v>
       </c>
       <c r="D15" s="40" t="n">
@@ -2990,54 +3045,54 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C16" s="40" t="n">
-        <f aca="false">Revenue!C8*Assumptions!C43/1000</f>
+        <f aca="false">Revenue!C8*Assumptions!C47/1000</f>
         <v>630</v>
       </c>
       <c r="D16" s="40" t="n">
-        <f aca="false">Revenue!D8*Assumptions!D43/1000</f>
+        <f aca="false">Revenue!D8*Assumptions!D47/1000</f>
         <v>705.6</v>
       </c>
       <c r="E16" s="40" t="n">
-        <f aca="false">Revenue!E8*Assumptions!E43/1000</f>
+        <f aca="false">Revenue!E8*Assumptions!E47/1000</f>
         <v>790.272</v>
       </c>
       <c r="F16" s="40" t="n">
-        <f aca="false">Revenue!F8*Assumptions!F43/1000</f>
+        <f aca="false">Revenue!F8*Assumptions!F47/1000</f>
         <v>885.10464</v>
       </c>
       <c r="G16" s="40" t="n">
-        <f aca="false">Revenue!G8*Assumptions!G43/1000</f>
+        <f aca="false">Revenue!G8*Assumptions!G47/1000</f>
         <v>1013.00226048</v>
       </c>
       <c r="H16" s="40" t="n">
-        <f aca="false">Revenue!H8*Assumptions!H43/1000</f>
+        <f aca="false">Revenue!H8*Assumptions!H47/1000</f>
         <v>1104.1724639232</v>
       </c>
       <c r="I16" s="40" t="n">
-        <f aca="false">Revenue!I8*Assumptions!I43/1000</f>
+        <f aca="false">Revenue!I8*Assumptions!I47/1000</f>
         <v>1203.54798567629</v>
       </c>
       <c r="J16" s="40" t="n">
-        <f aca="false">Revenue!J8*Assumptions!J43/1000</f>
+        <f aca="false">Revenue!J8*Assumptions!J47/1000</f>
         <v>1311.86730438715</v>
       </c>
       <c r="K16" s="40" t="n">
-        <f aca="false">Revenue!K8*Assumptions!K43/1000</f>
+        <f aca="false">Revenue!K8*Assumptions!K47/1000</f>
         <v>1473.88291647897</v>
       </c>
       <c r="L16" s="40" t="n">
-        <f aca="false">Revenue!L8*Assumptions!L43/1000</f>
+        <f aca="false">Revenue!L8*Assumptions!L47/1000</f>
         <v>1577.0547206325</v>
       </c>
       <c r="M16" s="40" t="n">
-        <f aca="false">Revenue!M8*Assumptions!M43/1000</f>
+        <f aca="false">Revenue!M8*Assumptions!M47/1000</f>
         <v>1687.44855107677</v>
       </c>
       <c r="N16" s="40" t="n">
-        <f aca="false">Revenue!N8*Assumptions!N43/1000</f>
+        <f aca="false">Revenue!N8*Assumptions!N47/1000</f>
         <v>1805.56994965214</v>
       </c>
       <c r="O16" s="41" t="n">
@@ -3047,54 +3102,54 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C17" s="40" t="n">
-        <f aca="false">C15*Assumptions!C45</f>
+        <f aca="false">C15*Assumptions!C49</f>
         <v>117.994201512732</v>
       </c>
       <c r="D17" s="40" t="n">
-        <f aca="false">D15*Assumptions!D45</f>
+        <f aca="false">D15*Assumptions!D49</f>
         <v>157.58810879181</v>
       </c>
       <c r="E17" s="40" t="n">
-        <f aca="false">E15*Assumptions!E45</f>
+        <f aca="false">E15*Assumptions!E49</f>
         <v>202.837690503039</v>
       </c>
       <c r="F17" s="40" t="n">
-        <f aca="false">F15*Assumptions!F45</f>
+        <f aca="false">F15*Assumptions!F49</f>
         <v>254.453786500175</v>
       </c>
       <c r="G17" s="40" t="n">
-        <f aca="false">G15*Assumptions!G45</f>
+        <f aca="false">G15*Assumptions!G49</f>
         <v>313.233680928827</v>
       </c>
       <c r="H17" s="40" t="n">
-        <f aca="false">H15*Assumptions!H45</f>
+        <f aca="false">H15*Assumptions!H49</f>
         <v>381.28995038041</v>
       </c>
       <c r="I17" s="40" t="n">
-        <f aca="false">I15*Assumptions!I45</f>
+        <f aca="false">I15*Assumptions!I49</f>
         <v>456.888815264788</v>
       </c>
       <c r="J17" s="40" t="n">
-        <f aca="false">J15*Assumptions!J45</f>
+        <f aca="false">J15*Assumptions!J49</f>
         <v>540.759513852907</v>
       </c>
       <c r="K17" s="40" t="n">
-        <f aca="false">K15*Assumptions!K45</f>
+        <f aca="false">K15*Assumptions!K49</f>
         <v>633.698708153625</v>
       </c>
       <c r="L17" s="40" t="n">
-        <f aca="false">L15*Assumptions!L45</f>
+        <f aca="false">L15*Assumptions!L49</f>
         <v>739.045928459163</v>
       </c>
       <c r="M17" s="40" t="n">
-        <f aca="false">M15*Assumptions!M45</f>
+        <f aca="false">M15*Assumptions!M49</f>
         <v>853.936081195144</v>
       </c>
       <c r="N17" s="40" t="n">
-        <f aca="false">N15*Assumptions!N45</f>
+        <f aca="false">N15*Assumptions!N49</f>
         <v>979.114283836442</v>
       </c>
       <c r="O17" s="41" t="n">
@@ -3104,54 +3159,54 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C18" s="40" t="n">
-        <f aca="false">-C15*Assumptions!C44</f>
+        <f aca="false">-C15*Assumptions!C48</f>
         <v>-43.3222411953254</v>
       </c>
       <c r="D18" s="40" t="n">
-        <f aca="false">-D15*Assumptions!D44</f>
+        <f aca="false">-D15*Assumptions!D48</f>
         <v>-57.8593691136366</v>
       </c>
       <c r="E18" s="40" t="n">
-        <f aca="false">-E15*Assumptions!E44</f>
+        <f aca="false">-E15*Assumptions!E48</f>
         <v>-74.4730100192867</v>
       </c>
       <c r="F18" s="40" t="n">
-        <f aca="false">-F15*Assumptions!F44</f>
+        <f aca="false">-F15*Assumptions!F48</f>
         <v>-93.4241528015678</v>
       </c>
       <c r="G18" s="40" t="n">
-        <f aca="false">-G15*Assumptions!G44</f>
+        <f aca="false">-G15*Assumptions!G48</f>
         <v>-115.005524862457</v>
       </c>
       <c r="H18" s="40" t="n">
-        <f aca="false">-H15*Assumptions!H44</f>
+        <f aca="false">-H15*Assumptions!H48</f>
         <v>-139.992770695189</v>
       </c>
       <c r="I18" s="40" t="n">
-        <f aca="false">-I15*Assumptions!I44</f>
+        <f aca="false">-I15*Assumptions!I48</f>
         <v>-167.749323276804</v>
       </c>
       <c r="J18" s="40" t="n">
-        <f aca="false">-J15*Assumptions!J44</f>
+        <f aca="false">-J15*Assumptions!J48</f>
         <v>-198.542926579954</v>
       </c>
       <c r="K18" s="40" t="n">
-        <f aca="false">-K15*Assumptions!K44</f>
+        <f aca="false">-K15*Assumptions!K48</f>
         <v>-232.666079585573</v>
       </c>
       <c r="L18" s="40" t="n">
-        <f aca="false">-L15*Assumptions!L44</f>
+        <f aca="false">-L15*Assumptions!L48</f>
         <v>-271.344909806236</v>
       </c>
       <c r="M18" s="40" t="n">
-        <f aca="false">-M15*Assumptions!M44</f>
+        <f aca="false">-M15*Assumptions!M48</f>
         <v>-313.527481864736</v>
       </c>
       <c r="N18" s="40" t="n">
-        <f aca="false">-N15*Assumptions!N44</f>
+        <f aca="false">-N15*Assumptions!N48</f>
         <v>-359.487369873626</v>
       </c>
       <c r="O18" s="41" t="n">
@@ -3161,7 +3216,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C19" s="42" t="n">
         <f aca="false">C15+C16+C17+C18</f>
@@ -3218,7 +3273,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C20" s="40" t="n">
         <f aca="false">C19/12</f>
@@ -3271,7 +3326,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C21" s="41" t="n">
         <f aca="false">AVERAGE(C15,C19)/4</f>
@@ -3328,7 +3383,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C22" s="34" t="n">
         <f aca="false">C21*1000</f>
@@ -3413,7 +3468,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3433,7 +3488,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -3454,51 +3509,51 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="11"/>
       <c r="B4" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C4" s="31" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="K4" s="31" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="L4" s="10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="M4" s="10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="N4" s="10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="O4" s="10" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C5" s="43" t="n">
         <f aca="false">Revenue!C22</f>
@@ -3555,54 +3610,54 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C6" s="34" t="n">
-        <f aca="false">-C5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-C5*(1-Assumptions!$C$33)</f>
         <v>-134878.478908729</v>
       </c>
       <c r="D6" s="34" t="n">
-        <f aca="false">-D5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-D5*(1-Assumptions!$C$33)</f>
         <v>-176403.498158607</v>
       </c>
       <c r="E6" s="34" t="n">
-        <f aca="false">-E5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-E5*(1-Assumptions!$C$33)</f>
         <v>-223812.54721306</v>
       </c>
       <c r="F6" s="34" t="n">
-        <f aca="false">-F5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-F5*(1-Assumptions!$C$33)</f>
         <v>-277843.748453075</v>
       </c>
       <c r="G6" s="34" t="n">
-        <f aca="false">-G5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-G5*(1-Assumptions!$C$33)</f>
         <v>-339921.277434812</v>
       </c>
       <c r="H6" s="34" t="n">
-        <f aca="false">-H5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-H5*(1-Assumptions!$C$33)</f>
         <v>-410230.529089069</v>
       </c>
       <c r="I6" s="34" t="n">
-        <f aca="false">-I5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-I5*(1-Assumptions!$C$33)</f>
         <v>-488279.849924068</v>
       </c>
       <c r="J6" s="34" t="n">
-        <f aca="false">-J5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-J5*(1-Assumptions!$C$33)</f>
         <v>-574816.062580488</v>
       </c>
       <c r="K6" s="34" t="n">
-        <f aca="false">-K5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-K5*(1-Assumptions!$C$33)</f>
         <v>-671863.547089934</v>
       </c>
       <c r="L6" s="34" t="n">
-        <f aca="false">-L5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-L5*(1-Assumptions!$C$33)</f>
         <v>-779654.507409076</v>
       </c>
       <c r="M6" s="34" t="n">
-        <f aca="false">-M5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-M5*(1-Assumptions!$C$33)</f>
         <v>-897151.361875623</v>
       </c>
       <c r="N6" s="34" t="n">
-        <f aca="false">-N5*(1-Assumptions!$C$29)</f>
+        <f aca="false">-N5*(1-Assumptions!$C$33)</f>
         <v>-1025110.34726123</v>
       </c>
       <c r="O6" s="35" t="n">
@@ -3612,7 +3667,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C7" s="44" t="n">
         <f aca="false">C5+C6</f>
@@ -3669,7 +3724,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C8" s="45" t="n">
         <f aca="false">IFERROR(C7/C5,0)</f>
@@ -3726,54 +3781,54 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C9" s="34" t="n">
-        <f aca="false">-C5*Assumptions!C46</f>
+        <f aca="false">-C5*Assumptions!C50</f>
         <v>-294280.317619044</v>
       </c>
       <c r="D9" s="34" t="n">
-        <f aca="false">-D5*Assumptions!D46</f>
+        <f aca="false">-D5*Assumptions!D50</f>
         <v>-374675.198568281</v>
       </c>
       <c r="E9" s="34" t="n">
-        <f aca="false">-E5*Assumptions!E46</f>
+        <f aca="false">-E5*Assumptions!E50</f>
         <v>-462422.618208802</v>
       </c>
       <c r="F9" s="34" t="n">
-        <f aca="false">-F5*Assumptions!F46</f>
+        <f aca="false">-F5*Assumptions!F50</f>
         <v>-557983.726232208</v>
       </c>
       <c r="G9" s="34" t="n">
-        <f aca="false">-G5*Assumptions!G46</f>
+        <f aca="false">-G5*Assumptions!G50</f>
         <v>-662986.954335666</v>
       </c>
       <c r="H9" s="34" t="n">
-        <f aca="false">-H5*Assumptions!H46</f>
+        <f aca="false">-H5*Assumptions!H50</f>
         <v>-776386.703813196</v>
       </c>
       <c r="I9" s="34" t="n">
-        <f aca="false">-I5*Assumptions!I46</f>
+        <f aca="false">-I5*Assumptions!I50</f>
         <v>-895852.286637546</v>
       </c>
       <c r="J9" s="34" t="n">
-        <f aca="false">-J5*Assumptions!J46</f>
+        <f aca="false">-J5*Assumptions!J50</f>
         <v>-1021367.38392401</v>
       </c>
       <c r="K9" s="34" t="n">
-        <f aca="false">-K5*Assumptions!K46</f>
+        <f aca="false">-K5*Assumptions!K50</f>
         <v>-1154938.9900389</v>
       </c>
       <c r="L9" s="34" t="n">
-        <f aca="false">-L5*Assumptions!L46</f>
+        <f aca="false">-L5*Assumptions!L50</f>
         <v>-1295128.56189442</v>
       </c>
       <c r="M9" s="34" t="n">
-        <f aca="false">-M5*Assumptions!M46</f>
+        <f aca="false">-M5*Assumptions!M50</f>
         <v>-1438407.96862703</v>
       </c>
       <c r="N9" s="34" t="n">
-        <f aca="false">-N5*Assumptions!N46</f>
+        <f aca="false">-N5*Assumptions!N50</f>
         <v>-1584261.44576736</v>
       </c>
       <c r="O9" s="35" t="n">
@@ -3783,54 +3838,54 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C10" s="34" t="n">
-        <f aca="false">-C5*Assumptions!C47</f>
+        <f aca="false">-C5*Assumptions!C51</f>
         <v>-183925.198511903</v>
       </c>
       <c r="D10" s="34" t="n">
-        <f aca="false">-D5*Assumptions!D47</f>
+        <f aca="false">-D5*Assumptions!D51</f>
         <v>-234718.704161452</v>
       </c>
       <c r="E10" s="34" t="n">
-        <f aca="false">-E5*Assumptions!E47</f>
+        <f aca="false">-E5*Assumptions!E51</f>
         <v>-290401.404235128</v>
       </c>
       <c r="F10" s="34" t="n">
-        <f aca="false">-F5*Assumptions!F47</f>
+        <f aca="false">-F5*Assumptions!F51</f>
         <v>-351323.086886946</v>
       </c>
       <c r="G10" s="34" t="n">
-        <f aca="false">-G5*Assumptions!G47</f>
+        <f aca="false">-G5*Assumptions!G51</f>
         <v>-418580.746593281</v>
       </c>
       <c r="H10" s="34" t="n">
-        <f aca="false">-H5*Assumptions!H47</f>
+        <f aca="false">-H5*Assumptions!H51</f>
         <v>-491598.567916653</v>
       </c>
       <c r="I10" s="34" t="n">
-        <f aca="false">-I5*Assumptions!I47</f>
+        <f aca="false">-I5*Assumptions!I51</f>
         <v>-568987.263134657</v>
       </c>
       <c r="J10" s="34" t="n">
-        <f aca="false">-J5*Assumptions!J47</f>
+        <f aca="false">-J5*Assumptions!J51</f>
         <v>-650824.798128321</v>
       </c>
       <c r="K10" s="34" t="n">
-        <f aca="false">-K5*Assumptions!K47</f>
+        <f aca="false">-K5*Assumptions!K51</f>
         <v>-738494.642669101</v>
       </c>
       <c r="L10" s="34" t="n">
-        <f aca="false">-L5*Assumptions!L47</f>
+        <f aca="false">-L5*Assumptions!L51</f>
         <v>-831201.91285761</v>
       </c>
       <c r="M10" s="34" t="n">
-        <f aca="false">-M5*Assumptions!M47</f>
+        <f aca="false">-M5*Assumptions!M51</f>
         <v>-926809.258135974</v>
       </c>
       <c r="N10" s="34" t="n">
-        <f aca="false">-N5*Assumptions!N47</f>
+        <f aca="false">-N5*Assumptions!N51</f>
         <v>-1025110.34726123</v>
       </c>
       <c r="O10" s="35" t="n">
@@ -3840,54 +3895,54 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C11" s="34" t="n">
-        <f aca="false">-C5*Assumptions!C48</f>
+        <f aca="false">-C5*Assumptions!C52</f>
         <v>-85831.7593055546</v>
       </c>
       <c r="D11" s="34" t="n">
-        <f aca="false">-D5*Assumptions!D48</f>
+        <f aca="false">-D5*Assumptions!D52</f>
         <v>-109341.011255335</v>
       </c>
       <c r="E11" s="34" t="n">
-        <f aca="false">-E5*Assumptions!E48</f>
+        <f aca="false">-E5*Assumptions!E52</f>
         <v>-135027.40451697</v>
       </c>
       <c r="F11" s="34" t="n">
-        <f aca="false">-F5*Assumptions!F48</f>
+        <f aca="false">-F5*Assumptions!F52</f>
         <v>-163032.282150151</v>
       </c>
       <c r="G11" s="34" t="n">
-        <f aca="false">-G5*Assumptions!G48</f>
+        <f aca="false">-G5*Assumptions!G52</f>
         <v>-193839.406140513</v>
       </c>
       <c r="H11" s="34" t="n">
-        <f aca="false">-H5*Assumptions!H48</f>
+        <f aca="false">-H5*Assumptions!H52</f>
         <v>-227152.441727005</v>
       </c>
       <c r="I11" s="34" t="n">
-        <f aca="false">-I5*Assumptions!I48</f>
+        <f aca="false">-I5*Assumptions!I52</f>
         <v>-262299.092934417</v>
       </c>
       <c r="J11" s="34" t="n">
-        <f aca="false">-J5*Assumptions!J48</f>
+        <f aca="false">-J5*Assumptions!J52</f>
         <v>-299284.396219593</v>
       </c>
       <c r="K11" s="34" t="n">
-        <f aca="false">-K5*Assumptions!K48</f>
+        <f aca="false">-K5*Assumptions!K52</f>
         <v>-338708.069194099</v>
       </c>
       <c r="L11" s="34" t="n">
-        <f aca="false">-L5*Assumptions!L48</f>
+        <f aca="false">-L5*Assumptions!L52</f>
         <v>-380162.115182938</v>
       </c>
       <c r="M11" s="34" t="n">
-        <f aca="false">-M5*Assumptions!M48</f>
+        <f aca="false">-M5*Assumptions!M52</f>
         <v>-422625.021710004</v>
       </c>
       <c r="N11" s="34" t="n">
-        <f aca="false">-N5*Assumptions!N48</f>
+        <f aca="false">-N5*Assumptions!N52</f>
         <v>-465959.248755106</v>
       </c>
       <c r="O11" s="35" t="n">
@@ -3897,7 +3952,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C12" s="44" t="n">
         <f aca="false">SUM(C9:C11)</f>
@@ -3954,7 +4009,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C13" s="46" t="n">
         <f aca="false">C7+C12</f>
@@ -4011,7 +4066,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C14" s="45" t="n">
         <f aca="false">IFERROR(C13/C5,0)</f>
@@ -4068,7 +4123,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -4089,21 +4144,21 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11"/>
       <c r="B18" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E18" s="10" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C19" s="41" t="n">
         <f aca="false">SUM(C5:F5)/1000</f>
@@ -4120,7 +4175,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C20" s="41" t="n">
         <f aca="false">SUM(C7:F7)/1000</f>
@@ -4137,7 +4192,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C21" s="41" t="n">
         <f aca="false">SUM(C13:F13)/1000</f>

</xml_diff>